<commit_message>
feat(m10): add external portal access for entities
Implements US-M10-005 with portal user provisioning + read-only portal APIs, plus workbook status/remarks updates and supporting migrations/scripts.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/Client-PM-Input-Register.xlsx
+++ b/docs/Client-PM-Input-Register.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\HRSrini\gapmc-management-system\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harsh\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C95B0B10-C735-4391-9C27-FD94B57CA8A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27161723-B860-458B-A0C1-62D5C768269C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PM input register" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="61">
   <si>
     <t>#</t>
   </si>
@@ -164,16 +164,165 @@
   </si>
   <si>
     <t>PM Response</t>
+  </si>
+  <si>
+    <t>Access to the application is provided via username and password authentication.
+Once all forms within the application are submitted, accepted, approved by the client, and frozen, an additional layer of security will be implemented by enabling CAPTCHA verification.</t>
+  </si>
+  <si>
+    <t>In the current release, all receipts, reports, and other documents will be formatted for A4 page size and made available as PDF downloads.</t>
+  </si>
+  <si>
+    <t>Since the client is not technically equipped to make this decision, we need to provide the most suitable solution.</t>
+  </si>
+  <si>
+    <t>Digital signatures will not be implemented for signing any receipts or system-generated outputs in the current release. 
+A placeholder may be retained to allow for potential future enhancement requests from the client. However, since this functionality is not technically required, implementing it later should not pose significant difficulty if such a requirement arises.</t>
+  </si>
+  <si>
+    <r>
+      <t>System design must ensure it supports:
+Data Retention rules ( Should be permanent till the lifecycle of the application ) 
+Archival or deletion policies. (As the data grows if required we can recommend archival facility at their local storage and free server space )
+Audit/compliance requirements : All records to hold audit history</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> which has been already implemented in the current system good enough.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Which ledger accounts are used for each transaction, are menthoined </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Attached Excelsheet indicating the different Ledgers.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>posting timing (invoice vs receipt vs remittance), reversals; whether marginal first-month-over-threshold TDS applies. WILL UPDATE SEPARATELY</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">WILL UPDATE SEPARATELY, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The CSV format. For reports as output from out software application.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+Refer Attached Excelsheet indicating the different Ledgers.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep this functionally pending for Development </t>
+  </si>
+  <si>
+    <t>If a cheque provided by a premises holder is dishonoured, the amount recorded against the tax invoice is not accounted for and a reversal entry is passed. When the user generates a new tax invoice, interest is recalculated and reflected as arrears.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This entry would be make manually by the user. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep this functionally as currently released in the production Enviromment. No Changes </t>
+  </si>
+  <si>
+    <t xml:space="preserve">F.7 Pre-Receipt — Government / GST-Exempt Entity Rent Acknowledgement (M-02 / M-03)
+Issued: to Track B Government/GST-exempt entities on receipt of rent. A simple narrative acknowledgement — no GST, no itemized table, no GSTIN. Signed by Market Supervisor, [YARD NAME]. </t>
+  </si>
+  <si>
+    <t>Refer Attached Excelsheet indicating the different Ledgers.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -199,9 +348,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -210,6 +362,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF0000FF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -551,7 +708,7 @@
     <col min="3" max="3" width="10" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36.5" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="52.796875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="12.09765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="65" style="1" customWidth="1"/>
     <col min="7" max="16384" width="8.796875" style="1"/>
   </cols>
   <sheetData>
@@ -575,7 +732,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -591,8 +748,11 @@
       <c r="E2" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="F2" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="109.2" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -608,8 +768,11 @@
       <c r="E3" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="F3" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -624,6 +787,9 @@
       </c>
       <c r="E4" s="1" t="s">
         <v>15</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
@@ -642,8 +808,11 @@
       <c r="E5" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="F5" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="109.2" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -659,8 +828,11 @@
       <c r="E6" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="F6" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="124.8" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -676,8 +848,11 @@
       <c r="E7" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="F7" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -692,6 +867,9 @@
       </c>
       <c r="E8" s="1" t="s">
         <v>28</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
@@ -710,8 +888,11 @@
       <c r="E9" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="F9" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -726,6 +907,9 @@
       </c>
       <c r="E10" s="1" t="s">
         <v>34</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
@@ -744,6 +928,9 @@
       <c r="E11" s="1" t="s">
         <v>37</v>
       </c>
+      <c r="F11" s="1" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="12" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
@@ -761,6 +948,9 @@
       <c r="E12" s="1" t="s">
         <v>40</v>
       </c>
+      <c r="F12" s="2" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="13" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
@@ -778,8 +968,11 @@
       <c r="E13" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="F13" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="78" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -794,12 +987,15 @@
       </c>
       <c r="E14" s="1" t="s">
         <v>46</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E14" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E1 A6:E6 A5:D5 A4:D4 A2:C2 A3:D3 A8:E9 A7:D7 A11:D11 A10:D10 A14:C14 A12:D12 A13:D13" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Developer Remarks from  M01 to M10
</commit_message>
<xml_diff>
--- a/docs/Client-PM-Input-Register.xlsx
+++ b/docs/Client-PM-Input-Register.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harsh\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\HRSrini\gapmc-management-system\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27161723-B860-458B-A0C1-62D5C768269C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6E3AD12-7CDA-4F9D-A513-4E94440B51F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PM input register" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="75">
   <si>
     <t>#</t>
   </si>
@@ -37,6 +37,12 @@
     <t>What GAPLMB must provide (deliverable)</t>
   </si>
   <si>
+    <t>PM Response</t>
+  </si>
+  <si>
+    <t>Developer Remarks</t>
+  </si>
+  <si>
     <t>P2</t>
   </si>
   <si>
@@ -49,6 +55,12 @@
     <t>Official letterhead assets (logo, layout rules) per clarification Q48; files for pre-printed or body-only PDF use.</t>
   </si>
   <si>
+    <t>In the current release, all receipts, reports, and other documents will be formatted for A4 page size and made available as PDF downloads.</t>
+  </si>
+  <si>
+    <t>MATCH: PDFs are generated as A4 and downloadable. Receipt PDF supports branding logo + body-only/preprinted modes (server/receipt-pdf.ts). No further action required unless official letterhead assets/layout rules are provided.</t>
+  </si>
+  <si>
     <t>P0</t>
   </si>
   <si>
@@ -59,262 +71,198 @@
   </si>
   <si>
     <t>IdP choice (OIDC or SAML); tenant URLs; client ID/secret or certs; redirect URIs per env; attribute mapping to app users/roles; MFA policy; UAT test users.</t>
-  </si>
-  <si>
-    <t>#15</t>
-  </si>
-  <si>
-    <t>§6.1 FR-RENT-005 — TDS + GL</t>
-  </si>
-  <si>
-    <t>Signed GL rules: accounts, Dr/Cr, posting timing (invoice vs receipt vs remittance), reversals; whether marginal first-month-over-threshold TDS applies.</t>
-  </si>
-  <si>
-    <t>#33</t>
-  </si>
-  <si>
-    <t>§15.1 — Object storage / encryption</t>
-  </si>
-  <si>
-    <t>Approved cloud object store (or NIC S3-compatible); bucket/region; IAM; SSE-S3 vs KMS requirement; cutover window and approval for disk→bucket migration.</t>
-  </si>
-  <si>
-    <t>§8.6 DSC</t>
-  </si>
-  <si>
-    <t>FR-PRT-001 — Digital signature</t>
-  </si>
-  <si>
-    <t>Policy: class of DSC/HSM, which documents must be signed, approved CA/vendor, authorised signatories.</t>
-  </si>
-  <si>
-    <t>P1</t>
-  </si>
-  <si>
-    <t>#50</t>
-  </si>
-  <si>
-    <t>§16.2 — Data retention</t>
-  </si>
-  <si>
-    <t>Legal/compliance stance: archive-only vs purge allowed; formal retention years per module if different from defaults; session/login retention when applicable.</t>
-  </si>
-  <si>
-    <t>#49</t>
-  </si>
-  <si>
-    <t>§8.3 FR-RCP-008 — Tally export</t>
-  </si>
-  <si>
-    <t>Finance UAT: import CSV/XML in Tally Prime (or agreed tool); signed list of gaps or sign-off.</t>
-  </si>
-  <si>
-    <t>#17</t>
-  </si>
-  <si>
-    <t>§6.1 FR-RENT-003 — GSTR-1</t>
-  </si>
-  <si>
-    <t>Target filing software; sample required JSON or CA checklist; POS/state code rules beyond current export placeholders.</t>
-  </si>
-  <si>
-    <t>#16</t>
-  </si>
-  <si>
-    <t>FR-RENT-007 — Arrears / interest GL</t>
-  </si>
-  <si>
-    <t>GL rules to post dishonour interest (heads, timing, amount basis).</t>
-  </si>
-  <si>
-    <t>#31</t>
-  </si>
-  <si>
-    <t>BR-AST-35 / BR-RCP-34 — Dishonour bank charge</t>
-  </si>
-  <si>
-    <t>Confirm auto bank-charge voucher: yes/no; default amount source; expenditure head / narrative for voucher line.</t>
-  </si>
-  <si>
-    <t>#28–30</t>
-  </si>
-  <si>
-    <t>§8.3 FR-RCP-006 — 38 Tally heads</t>
-  </si>
-  <si>
-    <t>Process owner when live chart ≠ 38: who (DA) corrects master data; target chart approval.</t>
-  </si>
-  <si>
-    <t>#39–40</t>
-  </si>
-  <si>
-    <t>§10.1 FR-VEH — Fleet SLA</t>
-  </si>
-  <si>
-    <t>Business rules for full BR-VEH parity: calendar SLA, alerts, escalation (beyond maintenance-due + digest).</t>
-  </si>
-  <si>
-    <t>#18–19</t>
-  </si>
-  <si>
-    <t>§5.2 / §5.5 — Allottee / Pre-receipt</t>
-  </si>
-  <si>
-    <t>Confirm flows vs SRS appendix with BA; any GAPLMB-specific exceptions in writing.</t>
-  </si>
-  <si>
-    <t>PM Response</t>
   </si>
   <si>
     <t>Access to the application is provided via username and password authentication.
 Once all forms within the application are submitted, accepted, approved by the client, and frozen, an additional layer of security will be implemented by enabling CAPTCHA verification.</t>
   </si>
   <si>
-    <t>In the current release, all receipts, reports, and other documents will be formatted for A4 page size and made available as PDF downloads.</t>
+    <t>PARTIAL/DIFF: App uses username/password. No CAPTCHA implementation found; MFA exists (server/routes-auth.ts + MFA routes) but SSO not implemented. Action needed only if CAPTCHA/SSO/MFA policy is confirmed.</t>
+  </si>
+  <si>
+    <t>#15</t>
+  </si>
+  <si>
+    <t>§6.1 FR-RENT-005 — TDS + GL</t>
+  </si>
+  <si>
+    <t>Signed GL rules: accounts, Dr/Cr, posting timing (invoice vs receipt vs remittance), reversals; whether marginal first-month-over-threshold TDS applies.</t>
+  </si>
+  <si>
+    <t>Which ledger accounts are used for each transaction, are menthoined Attached Excelsheet indicating the different Ledgers.
+posting timing (invoice vs receipt vs remittance), reversals; whether marginal first-month-over-threshold TDS applies. WILL UPDATE SEPARATELY</t>
+  </si>
+  <si>
+    <t>PARTIAL: TDS fields exist for rent invoices/receipts, but GL posting timing/reversal rules are not specified here (response says will update separately). Cannot implement GL rules without structured mapping + timing decisions.</t>
+  </si>
+  <si>
+    <t>#33</t>
+  </si>
+  <si>
+    <t>§15.1 — Object storage / encryption</t>
+  </si>
+  <si>
+    <t>Approved cloud object store (or NIC S3-compatible); bucket/region; IAM; SSE-S3 vs KMS requirement; cutover window and approval for disk→bucket migration.</t>
   </si>
   <si>
     <t>Since the client is not technically equipped to make this decision, we need to provide the most suitable solution.</t>
+  </si>
+  <si>
+    <t>MATCH: Upload storage abstraction supports local or S3-compatible object storage with optional SSE=AES256 (server/object-storage.ts). No further action required unless client chooses S3 bucket/IAM/KMS specifics.</t>
+  </si>
+  <si>
+    <t>§8.6 DSC</t>
+  </si>
+  <si>
+    <t>FR-PRT-001 — Digital signature</t>
+  </si>
+  <si>
+    <t>Policy: class of DSC/HSM, which documents must be signed, approved CA/vendor, authorised signatories.</t>
   </si>
   <si>
     <t>Digital signatures will not be implemented for signing any receipts or system-generated outputs in the current release. 
 A placeholder may be retained to allow for potential future enhancement requests from the client. However, since this functionality is not technically required, implementing it later should not pose significant difficulty if such a requirement arises.</t>
   </si>
   <si>
-    <r>
-      <t>System design must ensure it supports:
+    <t>MATCH: No digital signature/DSC signing implemented (as per PM response). Placeholder only; no further action required for current release.</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>#50</t>
+  </si>
+  <si>
+    <t>§16.2 — Data retention</t>
+  </si>
+  <si>
+    <t>Legal/compliance stance: archive-only vs purge allowed; formal retention years per module if different from defaults; session/login retention when applicable.</t>
+  </si>
+  <si>
+    <t>System design must ensure it supports:
 Data Retention rules ( Should be permanent till the lifecycle of the application ) 
 Archival or deletion policies. (As the data grows if required we can recommend archival facility at their local storage and free server space )
-Audit/compliance requirements : All records to hold audit history</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> which has been already implemented in the current system good enough.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Which ledger accounts are used for each transaction, are menthoined </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Attached Excelsheet indicating the different Ledgers.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>posting timing (invoice vs receipt vs remittance), reversals; whether marginal first-month-over-threshold TDS applies. WILL UPDATE SEPARATELY</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">WILL UPDATE SEPARATELY, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>The CSV format. For reports as output from out software application.</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> 
+Audit/compliance requirements : All records to hold audit history which has been already implemented in the current system good enough.</t>
+  </si>
+  <si>
+    <t>MATCH: Data retention is treated as non-deleting; a retention audit/visibility job exists and does not purge data (server/data-retention-audit.ts). No further action required unless client mandates purge/archive workflows.</t>
+  </si>
+  <si>
+    <t>#49</t>
+  </si>
+  <si>
+    <t>§8.3 FR-RCP-008 — Tally export</t>
+  </si>
+  <si>
+    <t>Finance UAT: import CSV/XML in Tally Prime (or agreed tool); signed list of gaps or sign-off.</t>
+  </si>
+  <si>
+    <t>WILL UPDATE SEPARATELY, The CSV format. For reports as output from out software application. 
 Refer Attached Excelsheet indicating the different Ledgers.</t>
-    </r>
+  </si>
+  <si>
+    <t>PARTIAL: Tally export (CSV/XML) exists (server/routes-reports.ts) with ledger mapping tables. PM response says CSV format will be updated separately; ledger workbook is name list, not full transaction→ledger posting spec. Await final format/UAT sign-off.</t>
+  </si>
+  <si>
+    <t>#17</t>
+  </si>
+  <si>
+    <t>§6.1 FR-RENT-003 — GSTR-1</t>
+  </si>
+  <si>
+    <t>Target filing software; sample required JSON or CA checklist; POS/state code rules beyond current export placeholders.</t>
   </si>
   <si>
     <t xml:space="preserve">Keep this functionally pending for Development </t>
   </si>
   <si>
+    <t>DIFF: PM says keep pending, but GSTR-1 export is already implemented (GET /api/ioms/rent/gstr1) and UI supports CSV export (client/src/pages/rent/IomsRentInvoices.tsx). Decide whether to keep as delivered or disable.</t>
+  </si>
+  <si>
+    <t>#16</t>
+  </si>
+  <si>
+    <t>FR-RENT-007 — Arrears / interest GL</t>
+  </si>
+  <si>
+    <t>GL rules to post dishonour interest (heads, timing, amount basis).</t>
+  </si>
+  <si>
     <t>If a cheque provided by a premises holder is dishonoured, the amount recorded against the tax invoice is not accounted for and a reversal entry is passed. When the user generates a new tax invoice, interest is recalculated and reflected as arrears.</t>
   </si>
   <si>
+    <t>MATCH: Cheque dishonour/reversal triggers rent ledger recording + interest recomputation hint; arrears interest cron posts ongoing interest (server/routes-receipts-ioms.ts, server/cron-m03-rent-arrears-interest.ts). No further action required.</t>
+  </si>
+  <si>
+    <t>#31</t>
+  </si>
+  <si>
+    <t>BR-AST-35 / BR-RCP-34 — Dishonour bank charge</t>
+  </si>
+  <si>
+    <t>Confirm auto bank-charge voucher: yes/no; default amount source; expenditure head / narrative for voucher line.</t>
+  </si>
+  <si>
     <t xml:space="preserve">This entry would be make manually by the user. </t>
   </si>
   <si>
+    <t>MATCH: Dishonour bank charge is referenced as config hint only and is not auto-posted; aligns with manual entry instruction. No further action required.</t>
+  </si>
+  <si>
+    <t>#28–30</t>
+  </si>
+  <si>
+    <t>§8.3 FR-RCP-006 — 38 Tally heads</t>
+  </si>
+  <si>
+    <t>Process owner when live chart ≠ 38: who (DA) corrects master data; target chart approval.</t>
+  </si>
+  <si>
+    <t>Refer Attached Excelsheet indicating the different Ledgers.</t>
+  </si>
+  <si>
+    <t>NEEDS INPUT: System has tally ledger master + revenue-head mapping tables, but this response only points to ledger list. To implement 38-head compliance, need a structured mapping (revenue head / voucher kind / DrCr / ledger) and process owner rules.</t>
+  </si>
+  <si>
+    <t>#39–40</t>
+  </si>
+  <si>
+    <t>§10.1 FR-VEH — Fleet SLA</t>
+  </si>
+  <si>
+    <t>Business rules for full BR-VEH parity: calendar SLA, alerts, escalation (beyond maintenance-due + digest).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Keep this functionally as currently released in the production Enviromment. No Changes </t>
+  </si>
+  <si>
+    <t>MATCH: Scope confirmation (no changes). Current fleet alerts/reports remain as implemented. No further action required.</t>
+  </si>
+  <si>
+    <t>#18–19</t>
+  </si>
+  <si>
+    <t>§5.2 / §5.5 — Allottee / Pre-receipt</t>
+  </si>
+  <si>
+    <t>Confirm flows vs SRS appendix with BA; any GAPLMB-specific exceptions in writing.</t>
   </si>
   <si>
     <t xml:space="preserve">F.7 Pre-Receipt — Government / GST-Exempt Entity Rent Acknowledgement (M-02 / M-03)
 Issued: to Track B Government/GST-exempt entities on receipt of rent. A simple narrative acknowledgement — no GST, no itemized table, no GSTIN. Signed by Market Supervisor, [YARD NAME]. </t>
   </si>
   <si>
-    <t>Refer Attached Excelsheet indicating the different Ledgers.</t>
+    <t>PARTIAL: Pre-receipt flow exists for Track-B Govt sub-type entities (server/routes-traders-assets.ts). PM response mentions narrative acknowledgement output; need confirmation whether a pre-receipt PDF/letter format is required (no dedicated pre-receipt PDF generator located in this pass).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -353,7 +301,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -362,11 +310,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
-  <colors>
-    <mruColors>
-      <color rgb="FF0000FF"/>
-    </mruColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -700,7 +643,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.8984375" style="1" bestFit="1" customWidth="1"/>
@@ -709,10 +652,11 @@
     <col min="4" max="4" width="36.5" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="52.796875" style="1" customWidth="1"/>
     <col min="6" max="6" width="65" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.796875" style="1"/>
+    <col min="7" max="7" width="57.296875" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -729,273 +673,312 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="109.2" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="109.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="93.6" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="93.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="109.2" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="109.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="124.8" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="124.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="46.8" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="62.4" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="62.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>36</v>
+        <v>56</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>39</v>
+        <v>61</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="78" x14ac:dyDescent="0.3">
+        <v>68</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="78" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>44</v>
+        <v>70</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>46</v>
+        <v>72</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>59</v>
+        <v>73</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:E1 A6:E6 A5:D5 A4:D4 A2:C2 A3:D3 A8:E9 A7:D7 A11:D11 A10:D10 A14:C14 A12:D12 A13:D13" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>